<commit_message>
Added Day 3 Notes and Complete 3-Day Summary
</commit_message>
<xml_diff>
--- a/Databricks_Learning/Databricks 3-Day Beginner Study Plan  |  Data Engineering Foundation/Databricks_3Day_Beginner_Plan.xlsx
+++ b/Databricks_Learning/Databricks 3-Day Beginner Study Plan  |  Data Engineering Foundation/Databricks_3Day_Beginner_Plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pareshranjanrout/Downloads/Databricks 3-Day Beginner Study Plan  |  Data Engineering Foundation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10145130-6A81-0E42-A80F-86A268DE332B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE39B83-73CA-8C4D-868A-777384A0EB46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="151">
   <si>
     <t>Databricks 3-Day Beginner Study Plan  |  Data Engineering Foundation</t>
   </si>
@@ -549,12 +549,15 @@
   <si>
     <t>Done</t>
   </si>
+  <si>
+    <t>Pending</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -648,6 +651,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <i/>
       <sz val="12"/>
       <color rgb="FF555555"/>
@@ -655,7 +666,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -719,11 +730,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF9E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
@@ -741,6 +747,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -884,7 +908,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -892,34 +916,34 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -961,11 +985,56 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -980,40 +1049,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1325,26 +1360,26 @@
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
     </row>
     <row r="3" spans="2:6" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="2:6" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="6" spans="2:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -1360,9 +1395,10 @@
       <c r="E6" s="13" t="s">
         <v>5</v>
       </c>
+      <c r="F6" s="26"/>
     </row>
     <row r="7" spans="2:6" ht="70" x14ac:dyDescent="0.2">
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="37" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="14" t="s">
@@ -1374,12 +1410,12 @@
       <c r="E7" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="45" t="s">
+      <c r="F7" s="27" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="42" x14ac:dyDescent="0.2">
-      <c r="B8" s="35"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="16" t="s">
         <v>10</v>
       </c>
@@ -1389,10 +1425,10 @@
       <c r="E8" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="45"/>
+      <c r="F8" s="27"/>
     </row>
     <row r="9" spans="2:6" ht="56" x14ac:dyDescent="0.2">
-      <c r="B9" s="35"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="14" t="s">
         <v>13</v>
       </c>
@@ -1402,10 +1438,10 @@
       <c r="E9" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="45"/>
+      <c r="F9" s="27"/>
     </row>
     <row r="10" spans="2:6" ht="70" x14ac:dyDescent="0.2">
-      <c r="B10" s="36"/>
+      <c r="B10" s="39"/>
       <c r="C10" s="16" t="s">
         <v>16</v>
       </c>
@@ -1415,10 +1451,10 @@
       <c r="E10" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="45"/>
+      <c r="F10" s="27"/>
     </row>
     <row r="11" spans="2:6" ht="56" x14ac:dyDescent="0.2">
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="40" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="18" t="s">
@@ -1430,9 +1466,12 @@
       <c r="E11" s="19" t="s">
         <v>22</v>
       </c>
+      <c r="F11" s="27" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="12" spans="2:6" ht="84" x14ac:dyDescent="0.2">
-      <c r="B12" s="38"/>
+      <c r="B12" s="41"/>
       <c r="C12" s="20" t="s">
         <v>23</v>
       </c>
@@ -1442,9 +1481,10 @@
       <c r="E12" s="21" t="s">
         <v>25</v>
       </c>
+      <c r="F12" s="27"/>
     </row>
     <row r="13" spans="2:6" ht="84" x14ac:dyDescent="0.2">
-      <c r="B13" s="38"/>
+      <c r="B13" s="41"/>
       <c r="C13" s="18" t="s">
         <v>26</v>
       </c>
@@ -1454,9 +1494,10 @@
       <c r="E13" s="19" t="s">
         <v>28</v>
       </c>
+      <c r="F13" s="27"/>
     </row>
     <row r="14" spans="2:6" ht="70" x14ac:dyDescent="0.2">
-      <c r="B14" s="39"/>
+      <c r="B14" s="42"/>
       <c r="C14" s="20" t="s">
         <v>29</v>
       </c>
@@ -1466,9 +1507,10 @@
       <c r="E14" s="21" t="s">
         <v>31</v>
       </c>
+      <c r="F14" s="27"/>
     </row>
     <row r="15" spans="2:6" ht="70" x14ac:dyDescent="0.2">
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="43" t="s">
         <v>32</v>
       </c>
       <c r="C15" s="22" t="s">
@@ -1480,9 +1522,12 @@
       <c r="E15" s="23" t="s">
         <v>35</v>
       </c>
+      <c r="F15" s="28" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="16" spans="2:6" ht="70" x14ac:dyDescent="0.2">
-      <c r="B16" s="41"/>
+      <c r="B16" s="44"/>
       <c r="C16" s="24" t="s">
         <v>36</v>
       </c>
@@ -1492,9 +1537,10 @@
       <c r="E16" s="25" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" ht="70" x14ac:dyDescent="0.2">
-      <c r="B17" s="41"/>
+      <c r="F16" s="29"/>
+    </row>
+    <row r="17" spans="2:6" ht="70" x14ac:dyDescent="0.2">
+      <c r="B17" s="44"/>
       <c r="C17" s="22" t="s">
         <v>39</v>
       </c>
@@ -1504,9 +1550,10 @@
       <c r="E17" s="23" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" ht="70" x14ac:dyDescent="0.2">
-      <c r="B18" s="42"/>
+      <c r="F17" s="29"/>
+    </row>
+    <row r="18" spans="2:6" ht="70" x14ac:dyDescent="0.2">
+      <c r="B18" s="45"/>
       <c r="C18" s="24" t="s">
         <v>42</v>
       </c>
@@ -1516,18 +1563,21 @@
       <c r="E18" s="25" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="26" t="s">
+      <c r="F18" s="30"/>
+    </row>
+    <row r="20" spans="2:6" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="31" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="F7:F10"/>
+    <mergeCell ref="F11:F14"/>
+    <mergeCell ref="F15:F18"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B4:E4"/>
@@ -1552,17 +1602,17 @@
   <sheetData>
     <row r="1" spans="2:3" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="30"/>
+      <c r="C2" s="47"/>
     </row>
     <row r="4" spans="2:3" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="30"/>
+      <c r="C5" s="47"/>
     </row>
     <row r="6" spans="2:3" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
@@ -1638,10 +1688,10 @@
     </row>
     <row r="15" spans="2:3" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="16" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="C16" s="30"/>
+      <c r="C16" s="47"/>
     </row>
     <row r="17" spans="2:3" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="7" t="s">
@@ -1709,10 +1759,10 @@
     </row>
     <row r="25" spans="2:3" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="26" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="33" t="s">
+      <c r="B26" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="C26" s="30"/>
+      <c r="C26" s="47"/>
     </row>
     <row r="27" spans="2:3" ht="58" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="9" t="s">
@@ -1793,11 +1843,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
     </row>
     <row r="4" spans="2:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">

</xml_diff>